<commit_message>
Engagement: quiz and poll answers designed into the stories (no white boxes), 2 new engagement posts, every post logo set to 12%
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/Fresh-Valley-Content-Plan.xlsx
+++ b/files/Fresh-Valley-Content-Plan.xlsx
@@ -3501,6 +3501,72 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1447800" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1101" name="Picture 101"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId101"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1447800" cy="1809750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1447800" cy="1809750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1102" name="Picture 102"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId102"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1447800" cy="1809750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3516,7 +3582,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1101" name="Picture 101"/>
+        <xdr:cNvPr id="1103" name="Picture 103"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3549,7 +3615,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1102" name="Picture 102"/>
+        <xdr:cNvPr id="1104" name="Picture 104"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3582,7 +3648,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1103" name="Picture 103"/>
+        <xdr:cNvPr id="1105" name="Picture 105"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3615,7 +3681,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1104" name="Picture 104"/>
+        <xdr:cNvPr id="1106" name="Picture 106"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3648,7 +3714,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1105" name="Picture 105"/>
+        <xdr:cNvPr id="1107" name="Picture 107"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3681,7 +3747,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1106" name="Picture 106"/>
+        <xdr:cNvPr id="1108" name="Picture 108"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3714,7 +3780,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1107" name="Picture 107"/>
+        <xdr:cNvPr id="1109" name="Picture 109"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3747,7 +3813,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1108" name="Picture 108"/>
+        <xdr:cNvPr id="1110" name="Picture 110"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3780,7 +3846,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1109" name="Picture 109"/>
+        <xdr:cNvPr id="1111" name="Picture 111"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3813,7 +3879,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1110" name="Picture 110"/>
+        <xdr:cNvPr id="1112" name="Picture 112"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3846,7 +3912,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1111" name="Picture 111"/>
+        <xdr:cNvPr id="1113" name="Picture 113"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3879,7 +3945,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1112" name="Picture 112"/>
+        <xdr:cNvPr id="1114" name="Picture 114"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3912,7 +3978,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1113" name="Picture 113"/>
+        <xdr:cNvPr id="1115" name="Picture 115"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3945,7 +4011,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1114" name="Picture 114"/>
+        <xdr:cNvPr id="1116" name="Picture 116"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3978,7 +4044,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1115" name="Picture 115"/>
+        <xdr:cNvPr id="1117" name="Picture 117"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4011,7 +4077,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1116" name="Picture 116"/>
+        <xdr:cNvPr id="1118" name="Picture 118"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4044,7 +4110,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1117" name="Picture 117"/>
+        <xdr:cNvPr id="1119" name="Picture 119"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4077,7 +4143,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1118" name="Picture 118"/>
+        <xdr:cNvPr id="1120" name="Picture 120"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4110,7 +4176,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1119" name="Picture 119"/>
+        <xdr:cNvPr id="1121" name="Picture 121"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4143,7 +4209,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1120" name="Picture 120"/>
+        <xdr:cNvPr id="1122" name="Picture 122"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4176,7 +4242,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1121" name="Picture 121"/>
+        <xdr:cNvPr id="1123" name="Picture 123"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4209,7 +4275,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1122" name="Picture 122"/>
+        <xdr:cNvPr id="1124" name="Picture 124"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4242,7 +4308,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1123" name="Picture 123"/>
+        <xdr:cNvPr id="1125" name="Picture 125"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4275,7 +4341,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1124" name="Picture 124"/>
+        <xdr:cNvPr id="1126" name="Picture 126"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4308,7 +4374,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1125" name="Picture 125"/>
+        <xdr:cNvPr id="1127" name="Picture 127"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4341,7 +4407,7 @@
     <xdr:ext cx="1219200" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1126" name="Picture 126"/>
+        <xdr:cNvPr id="1128" name="Picture 128"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4379,7 +4445,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1127" name="Picture 127"/>
+        <xdr:cNvPr id="1129" name="Picture 129"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4412,7 +4478,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1128" name="Picture 128"/>
+        <xdr:cNvPr id="1130" name="Picture 130"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4445,7 +4511,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1129" name="Picture 129"/>
+        <xdr:cNvPr id="1131" name="Picture 131"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4478,7 +4544,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1130" name="Picture 130"/>
+        <xdr:cNvPr id="1132" name="Picture 132"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4511,7 +4577,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1131" name="Picture 131"/>
+        <xdr:cNvPr id="1133" name="Picture 133"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4544,7 +4610,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1132" name="Picture 132"/>
+        <xdr:cNvPr id="1134" name="Picture 134"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4577,7 +4643,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1133" name="Picture 133"/>
+        <xdr:cNvPr id="1135" name="Picture 135"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4610,7 +4676,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1134" name="Picture 134"/>
+        <xdr:cNvPr id="1136" name="Picture 136"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4643,7 +4709,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1135" name="Picture 135"/>
+        <xdr:cNvPr id="1137" name="Picture 137"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4676,7 +4742,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1136" name="Picture 136"/>
+        <xdr:cNvPr id="1138" name="Picture 138"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4709,7 +4775,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1137" name="Picture 137"/>
+        <xdr:cNvPr id="1139" name="Picture 139"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4742,7 +4808,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1138" name="Picture 138"/>
+        <xdr:cNvPr id="1140" name="Picture 140"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4775,7 +4841,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1139" name="Picture 139"/>
+        <xdr:cNvPr id="1141" name="Picture 141"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4808,7 +4874,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1140" name="Picture 140"/>
+        <xdr:cNvPr id="1142" name="Picture 142"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4841,7 +4907,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1141" name="Picture 141"/>
+        <xdr:cNvPr id="1143" name="Picture 143"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4874,7 +4940,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1142" name="Picture 142"/>
+        <xdr:cNvPr id="1144" name="Picture 144"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4907,7 +4973,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1143" name="Picture 143"/>
+        <xdr:cNvPr id="1145" name="Picture 145"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4940,7 +5006,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1144" name="Picture 144"/>
+        <xdr:cNvPr id="1146" name="Picture 146"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -4973,7 +5039,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1145" name="Picture 145"/>
+        <xdr:cNvPr id="1147" name="Picture 147"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5006,7 +5072,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1146" name="Picture 146"/>
+        <xdr:cNvPr id="1148" name="Picture 148"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5039,7 +5105,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1147" name="Picture 147"/>
+        <xdr:cNvPr id="1149" name="Picture 149"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5072,7 +5138,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1148" name="Picture 148"/>
+        <xdr:cNvPr id="1150" name="Picture 150"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5105,7 +5171,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1149" name="Picture 149"/>
+        <xdr:cNvPr id="1151" name="Picture 151"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5138,7 +5204,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1150" name="Picture 150"/>
+        <xdr:cNvPr id="1152" name="Picture 152"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5171,7 +5237,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1151" name="Picture 151"/>
+        <xdr:cNvPr id="1153" name="Picture 153"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5204,7 +5270,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1152" name="Picture 152"/>
+        <xdr:cNvPr id="1154" name="Picture 154"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5237,7 +5303,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1153" name="Picture 153"/>
+        <xdr:cNvPr id="1155" name="Picture 155"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5270,7 +5336,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1154" name="Picture 154"/>
+        <xdr:cNvPr id="1156" name="Picture 156"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5303,7 +5369,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1155" name="Picture 155"/>
+        <xdr:cNvPr id="1157" name="Picture 157"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5336,7 +5402,7 @@
     <xdr:ext cx="1028700" cy="1828800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1156" name="Picture 156"/>
+        <xdr:cNvPr id="1158" name="Picture 158"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5374,7 +5440,7 @@
     <xdr:ext cx="4953000" cy="10086975"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1157" name="Picture 157"/>
+        <xdr:cNvPr id="1159" name="Picture 159"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5412,7 +5478,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1158" name="Picture 158"/>
+        <xdr:cNvPr id="1160" name="Picture 160"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5445,7 +5511,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1159" name="Picture 159"/>
+        <xdr:cNvPr id="1161" name="Picture 161"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5478,7 +5544,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1160" name="Picture 160"/>
+        <xdr:cNvPr id="1162" name="Picture 162"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5511,7 +5577,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1161" name="Picture 161"/>
+        <xdr:cNvPr id="1163" name="Picture 163"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5544,7 +5610,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1162" name="Picture 162"/>
+        <xdr:cNvPr id="1164" name="Picture 164"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5577,7 +5643,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1163" name="Picture 163"/>
+        <xdr:cNvPr id="1165" name="Picture 165"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5610,7 +5676,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1164" name="Picture 164"/>
+        <xdr:cNvPr id="1166" name="Picture 166"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5643,7 +5709,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1165" name="Picture 165"/>
+        <xdr:cNvPr id="1167" name="Picture 167"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5676,7 +5742,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1166" name="Picture 166"/>
+        <xdr:cNvPr id="1168" name="Picture 168"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5709,7 +5775,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1167" name="Picture 167"/>
+        <xdr:cNvPr id="1169" name="Picture 169"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5742,7 +5808,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1168" name="Picture 168"/>
+        <xdr:cNvPr id="1170" name="Picture 170"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5775,7 +5841,7 @@
     <xdr:ext cx="1905000" cy="2381250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1169" name="Picture 169"/>
+        <xdr:cNvPr id="1171" name="Picture 171"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5813,7 +5879,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1170" name="Picture 170"/>
+        <xdr:cNvPr id="1172" name="Picture 172"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5846,7 +5912,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1171" name="Picture 171"/>
+        <xdr:cNvPr id="1173" name="Picture 173"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5879,7 +5945,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1172" name="Picture 172"/>
+        <xdr:cNvPr id="1174" name="Picture 174"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5912,7 +5978,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1173" name="Picture 173"/>
+        <xdr:cNvPr id="1175" name="Picture 175"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5945,7 +6011,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1174" name="Picture 174"/>
+        <xdr:cNvPr id="1176" name="Picture 176"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -5978,7 +6044,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1175" name="Picture 175"/>
+        <xdr:cNvPr id="1177" name="Picture 177"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6011,7 +6077,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1176" name="Picture 176"/>
+        <xdr:cNvPr id="1178" name="Picture 178"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6044,7 +6110,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1177" name="Picture 177"/>
+        <xdr:cNvPr id="1179" name="Picture 179"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6077,7 +6143,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1178" name="Picture 178"/>
+        <xdr:cNvPr id="1180" name="Picture 180"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6110,7 +6176,7 @@
     <xdr:ext cx="2476500" cy="542925"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1179" name="Picture 179"/>
+        <xdr:cNvPr id="1181" name="Picture 181"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6143,7 +6209,7 @@
     <xdr:ext cx="2476500" cy="1485900"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1180" name="Picture 180"/>
+        <xdr:cNvPr id="1182" name="Picture 182"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6176,7 +6242,7 @@
     <xdr:ext cx="2476500" cy="561975"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1181" name="Picture 181"/>
+        <xdr:cNvPr id="1183" name="Picture 183"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6209,7 +6275,7 @@
     <xdr:ext cx="2476500" cy="561975"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1182" name="Picture 182"/>
+        <xdr:cNvPr id="1184" name="Picture 184"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6242,7 +6308,7 @@
     <xdr:ext cx="2476500" cy="561975"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1183" name="Picture 183"/>
+        <xdr:cNvPr id="1185" name="Picture 185"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6275,7 +6341,7 @@
     <xdr:ext cx="2476500" cy="561975"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1184" name="Picture 184"/>
+        <xdr:cNvPr id="1186" name="Picture 186"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6308,7 +6374,7 @@
     <xdr:ext cx="2476500" cy="561975"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1185" name="Picture 185"/>
+        <xdr:cNvPr id="1187" name="Picture 187"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6341,7 +6407,7 @@
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1186" name="Picture 186"/>
+        <xdr:cNvPr id="1188" name="Picture 188"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6372,7 +6438,7 @@
   <sheetPr>
     <tabColor rgb="FF19291C"/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -6410,7 +6476,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">100 posts · 20 weeks · Sun–Thu from Sunday 1 November 2026 · post in this exact order — dark / light alternate so the 3-column grid always reads as a checkerboard · carousels: see the Carousels tab</t>
+          <t xml:space="preserve">102 posts · 21 weeks · Sun–Thu from Sunday 1 November 2026 · post in this exact order — dark / light alternate so the 3-column grid always reads as a checkerboard · carousels: see the Carousels tab</t>
         </is>
       </c>
       <c r="B2" s="3"/>
@@ -12103,13 +12169,127 @@
         </is>
       </c>
     </row>
+    <row r="105" ht="152" customHeight="1">
+      <c r="A105" s="7">
+        <v>101</v>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dark</t>
+        </is>
+      </c>
+      <c r="C105" s="6"/>
+      <c r="D105" s="8">
+        <v>46467</v>
+      </c>
+      <c r="E105" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8:30 pm</t>
+        </is>
+      </c>
+      <c r="F105" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Table</t>
+        </is>
+      </c>
+      <c r="G105" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giant word + produce
+Engagement</t>
+        </is>
+      </c>
+      <c r="H105" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This or that? · Comment A or B.</t>
+        </is>
+      </c>
+      <c r="I105" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dates or figs — which one makes your table? Comment A or B.
+Order before noon — at your door today. Link in bio.</t>
+        </is>
+      </c>
+      <c r="J105" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تمر ولا تين — مين اللي بيكمّل سفرتك؟ اكتب A أو B.
+اطلب قبل الضهر — يوصلك النهارده. الرابط في البايو.</t>
+        </is>
+      </c>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+        </is>
+      </c>
+      <c r="L105" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="152" customHeight="1">
+      <c r="A106" s="7">
+        <v>102</v>
+      </c>
+      <c r="B106" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Light</t>
+        </is>
+      </c>
+      <c r="C106" s="6"/>
+      <c r="D106" s="8">
+        <v>46468</v>
+      </c>
+      <c r="E106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8:30 pm</t>
+        </is>
+      </c>
+      <c r="F106" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Living Well</t>
+        </is>
+      </c>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type statement
+Engagement</t>
+        </is>
+      </c>
+      <c r="H106" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True or false? Basil belongs in the fridge.</t>
+        </is>
+      </c>
+      <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True or false: basil belongs in the fridge? Comment your answer — we’ll reply with the right one. (Hint: it loves a sunny windowsill.)
+Order before noon — at your door today. Link in bio.</t>
+        </is>
+      </c>
+      <c r="J106" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">صح ولا غلط: الريحان مكانه التلاجة؟ اكتب إجابتك وهنرد عليك. (تلميح: بيحب الشباك والشمس.)
+اطلب قبل الضهر — يوصلك النهارده. الرابط في البايو.</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+        </is>
+      </c>
+      <c r="L106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ready</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5:L104">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5:L106">
       <formula1>"Ready,Scheduled,Posted"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12333,7 +12513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1080 × 1920 · files in social/stories · keep the top and bottom 250 px clear — the designs already do · add the sticker listed below where the design leaves space</t>
+          <t xml:space="preserve">1080 × 1920 · files in social/stories · keep the top and bottom 250 px clear — the designs already do · quizzes and polls have their answers designed in — no white boxes, no stickers needed</t>
         </is>
       </c>
       <c r="B2" s="3"/>
@@ -12377,7 +12557,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sticker to add</t>
+          <t xml:space="preserve">Sticker / answers</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -12479,7 +12659,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poll: “Tray” / “Bowl”</t>
+          <t xml:space="preserve">No sticker — the answers are in the design (A Tray / B Bowl). Replies arrive by DM.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -12683,7 +12863,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz: “One” / “A few” / “Every piece” (answer: Every piece)</t>
+          <t xml:space="preserve">No sticker — the answers are in the design (A One / B A few / C Every piece). Replies arrive by DM.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -12887,7 +13067,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poll: “Mango” / “Strawberries”</t>
+          <t xml:space="preserve">No sticker — the answers are in the design (A Mango / B Strawberries). Replies arrive by DM.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -12916,12 +13096,12 @@
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strawberry season starts soon.</t>
+          <t xml:space="preserve">When does strawberry season start?</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Countdown: “Strawberry season”</t>
+          <t xml:space="preserve">No sticker — the answers are in the design (A Winter / B Spring / C Summer). Replies arrive by DM.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -13057,7 +13237,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Question: “What goes in your lunchbox?”</t>
+          <t xml:space="preserve">Question sticker: “What goes in your lunchbox?”</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -13091,7 +13271,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emoji slider: 🥬</t>
+          <t xml:space="preserve">No sticker — the answers are in the design (1 / 2 / 3 / 4 / 5). Replies arrive by DM.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
@@ -13397,7 +13577,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poll: “Fruit” / “Veg” / “Herbs” / “All of it”</t>
+          <t xml:space="preserve">No sticker — the answers are in the design (A Orchard / B Market / C Garden / D Salad Table / E Host). Replies arrive by DM.</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
@@ -14439,7 +14619,7 @@
         </is>
       </c>
       <c r="E4" s="6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F4" s="6">
         <v>6</v>
@@ -14517,7 +14697,7 @@
         </is>
       </c>
       <c r="E7" s="6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" s="6">
         <v>6</v>

</xml_diff>

<commit_message>
Social: box and bag designs on the new packaging (contour lids, dividers, real logo); Facebook cover 1640x924
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/Fresh-Valley-Content-Plan.xlsx
+++ b/files/Fresh-Valley-Content-Plan.xlsx
@@ -6173,16 +6173,214 @@
       <xdr:row>13</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
+    <xdr:ext cx="2476500" cy="1619250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1181" name="Picture 181"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="1619250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="1619250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1182" name="Picture 182"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="1619250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="1619250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1183" name="Picture 183"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="1619250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="1619250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1184" name="Picture 184"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="1619250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="1619250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1185" name="Picture 185"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="1619250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="1619250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1186" name="Picture 186"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="1619250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
     <xdr:ext cx="2476500" cy="542925"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1181" name="Picture 181"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <xdr:cNvPr id="1187" name="Picture 187"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6203,19 +6401,19 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2476500" cy="1485900"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1182" name="Picture 182"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <xdr:cNvPr id="1188" name="Picture 188"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6236,27 +6434,27 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2476500" cy="561975"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1183" name="Picture 183"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2476500" cy="561975"/>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1189" name="Picture 189"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="742950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6269,27 +6467,27 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2476500" cy="561975"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1184" name="Picture 184"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2476500" cy="561975"/>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1190" name="Picture 190"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="742950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6302,27 +6500,27 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2476500" cy="561975"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1185" name="Picture 185"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2476500" cy="561975"/>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1191" name="Picture 191"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="742950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6335,27 +6533,27 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2476500" cy="561975"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1186" name="Picture 186"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2476500" cy="561975"/>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1192" name="Picture 192"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="742950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6368,27 +6566,27 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2476500" cy="561975"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1187" name="Picture 187"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2476500" cy="561975"/>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2476500" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1193" name="Picture 193"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476500" cy="742950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6401,19 +6599,19 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2476500" cy="1619250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1188" name="Picture 188"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <xdr:cNvPr id="1194" name="Picture 194"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6476,7 +6674,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">102 posts · 21 weeks · Sun–Thu from Sunday 1 November 2026 · post in this exact order — dark / light alternate so the 3-column grid always reads as a checkerboard · carousels: see the Carousels tab</t>
+          <t xml:space="preserve">102 posts · one a day from Sunday 1 November 2026 to 10 February 2027 · Cairo time · English captions only · post in this exact order — dark / light alternate so the 3-column grid always reads as a checkerboard · carousels: see the Carousels tab</t>
         </is>
       </c>
       <c r="B2" s="3"/>
@@ -6534,12 +6732,12 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caption (EN)</t>
+          <t xml:space="preserve">Caption (posted)</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caption (AR)</t>
+          <t xml:space="preserve">Arabic (reference — not posted)</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
@@ -6568,7 +6766,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -6589,7 +6787,7 @@
       <c r="I5" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Navel oranges, seedless and full of juice. Picked whole, washed and at your door today.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr">
@@ -6600,7 +6798,7 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -6624,7 +6822,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -6645,7 +6843,7 @@
       <c r="I6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Mango season. Picked at the right moment so it is ripe on arrival.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J6" s="9" t="inlineStr">
@@ -6656,7 +6854,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -6680,7 +6878,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -6701,7 +6899,7 @@
       <c r="I7" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Picked today. Colour and clean skin. Taste. Every lot passes all three before it leaves the farm.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
@@ -6712,7 +6910,7 @@
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -6736,7 +6934,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
@@ -6757,7 +6955,7 @@
       <c r="I8" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A tray of whole fruit says more than a box of sweets.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
@@ -6768,7 +6966,7 @@
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -6792,7 +6990,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
@@ -6813,7 +7011,7 @@
       <c r="I9" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Orchard box: mango, grapes, figs, pomegranates, oranges and peaches — each in its own well.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr">
@@ -6824,7 +7022,7 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -6844,11 +7042,11 @@
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="8">
-        <v>46334</v>
+        <v>46332</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
@@ -6869,7 +7067,7 @@
       <c r="I10" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Oranges, lemons, romaine and beetroot — this week’s colours, picked whole.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J10" s="9" t="inlineStr">
@@ -6880,7 +7078,7 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -6900,11 +7098,11 @@
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="8">
-        <v>46335</v>
+        <v>46333</v>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
@@ -6925,7 +7123,7 @@
       <c r="I11" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Mint cut the morning it ships. Still lively when it arrives.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
@@ -6936,7 +7134,7 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -6956,11 +7154,11 @@
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="8">
-        <v>46336</v>
+        <v>46334</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
@@ -6981,7 +7179,7 @@
       <c r="I12" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The host’s gesture: a box of whole fruit instead of sweets.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr">
@@ -6992,7 +7190,7 @@
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -7012,11 +7210,11 @@
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="8">
-        <v>46337</v>
+        <v>46335</v>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
@@ -7037,7 +7235,7 @@
       <c r="I13" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">From the farm to your door on the same day. Less time travelling, more time fresh.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
@@ -7048,7 +7246,7 @@
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -7068,11 +7266,11 @@
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="8">
-        <v>46338</v>
+        <v>46336</v>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F14" s="14" t="inlineStr">
@@ -7093,7 +7291,7 @@
       <c r="I14" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Every piece is checked by hand before it is packed. Not perfect? It does not go in your box.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J14" s="9" t="inlineStr">
@@ -7104,7 +7302,7 @@
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -7124,11 +7322,11 @@
       </c>
       <c r="C15" s="6"/>
       <c r="D15" s="8">
-        <v>46341</v>
+        <v>46337</v>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
@@ -7149,7 +7347,7 @@
       <c r="I15" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Tight green broccoli heads, cut the morning they ship.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr">
@@ -7160,7 +7358,7 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -7180,11 +7378,11 @@
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="8">
-        <v>46342</v>
+        <v>46338</v>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F16" s="15" t="inlineStr">
@@ -7205,7 +7403,7 @@
       <c r="I16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">What’s best in October: pomegranates, fresh dates, the last grapes and figs, okra and apples.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J16" s="9" t="inlineStr">
@@ -7216,7 +7414,7 @@
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -7236,11 +7434,11 @@
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="8">
-        <v>46343</v>
+        <v>46339</v>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -7261,7 +7459,7 @@
       <c r="I17" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">If anything isn’t right, send a photo on WhatsApp within 24 hours. We replace it or refund it.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
@@ -7272,7 +7470,7 @@
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -7292,11 +7490,11 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="8">
-        <v>46344</v>
+        <v>46340</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
@@ -7317,7 +7515,7 @@
       <c r="I18" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The host’s first gesture: a small bowl of Medjool dates by the door.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J18" s="9" t="inlineStr">
@@ -7328,7 +7526,7 @@
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -7348,11 +7546,11 @@
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="8">
-        <v>46345</v>
+        <v>46341</v>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F19" s="16" t="inlineStr">
@@ -7373,7 +7571,7 @@
       <c r="I19" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Basil, mint and parsley — cut to order, washed and bunched the morning they ship.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
@@ -7384,7 +7582,7 @@
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -7404,11 +7602,11 @@
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="8">
-        <v>46348</v>
+        <v>46342</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -7429,7 +7627,7 @@
       <c r="I20" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Zebdia mango — the one every Egyptian table asks for. Back from July to September.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
@@ -7440,7 +7638,7 @@
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -7460,11 +7658,11 @@
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="8">
-        <v>46349</v>
+        <v>46343</v>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -7485,7 +7683,7 @@
       <c r="I21" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Market box: fruit on one side, vegetables on the other. The week, sorted.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
@@ -7496,7 +7694,7 @@
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -7516,11 +7714,11 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="8">
-        <v>46350</v>
+        <v>46344</v>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr">
@@ -7541,7 +7739,7 @@
       <c r="I22" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Orchard: six fruits at their peak, each in its own well.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
@@ -7552,7 +7750,7 @@
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -7572,11 +7770,11 @@
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="8">
-        <v>46351</v>
+        <v>46345</v>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
@@ -7597,7 +7795,7 @@
       <c r="I23" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Pomegranates — heavy, deep red and delivered whole.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
@@ -7608,7 +7806,7 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -7628,11 +7826,11 @@
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="8">
-        <v>46352</v>
+        <v>46346</v>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr">
@@ -7653,7 +7851,7 @@
       <c r="I24" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Grapes, dates, strawberries and mint — the four things that make a tray.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J24" s="9" t="inlineStr">
@@ -7664,7 +7862,7 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
@@ -7684,11 +7882,11 @@
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="8">
-        <v>46355</v>
+        <v>46347</v>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
@@ -7709,7 +7907,7 @@
       <c r="I25" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A good cucumber snaps. Ours are picked young, crisp and thin-skinned.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr">
@@ -7720,7 +7918,7 @@
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -7740,11 +7938,11 @@
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="8">
-        <v>46356</v>
+        <v>46348</v>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F26" s="15" t="inlineStr">
@@ -7765,7 +7963,7 @@
       <c r="I26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Winter strawberries are back. Picked at full colour and chilled within hours.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr">
@@ -7776,7 +7974,7 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -7796,11 +7994,11 @@
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="8">
-        <v>46357</v>
+        <v>46349</v>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
@@ -7821,7 +8019,7 @@
       <c r="I27" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">We wash every piece by hand and never wax it. What you see is the fruit.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
@@ -7832,7 +8030,7 @@
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -7852,11 +8050,11 @@
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="8">
-        <v>46358</v>
+        <v>46350</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
@@ -7877,7 +8075,7 @@
       <c r="I28" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Our tomatoes ripen on the vine and are picked red. They taste like tomatoes again.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J28" s="9" t="inlineStr">
@@ -7888,7 +8086,7 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -7908,11 +8106,11 @@
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="8">
-        <v>46359</v>
+        <v>46351</v>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
@@ -7933,7 +8131,7 @@
       <c r="I29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Avocado, herbs and whatever is in season — breakfast that starts in the garden.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
@@ -7944,7 +8142,7 @@
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr">
@@ -7964,11 +8162,11 @@
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="8">
-        <v>46362</v>
+        <v>46352</v>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F30" s="16" t="inlineStr">
@@ -7989,7 +8187,7 @@
       <c r="I30" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Crisp romaine, cut this morning. The easiest way to eat more plants.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J30" s="9" t="inlineStr">
@@ -8000,7 +8198,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr">
@@ -8020,11 +8218,11 @@
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="8">
-        <v>46363</v>
+        <v>46353</v>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F31" s="17" t="inlineStr">
@@ -8045,7 +8243,7 @@
       <c r="I31" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Garden box: six herb bunches standing in sleeves, plus a jar of live basil.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr">
@@ -8056,7 +8254,7 @@
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr">
@@ -8076,11 +8274,11 @@
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="8">
-        <v>46364</v>
+        <v>46354</v>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F32" s="15" t="inlineStr">
@@ -8101,7 +8299,7 @@
       <c r="I32" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">November brings the first oranges and strawberries, guava, persimmon, cabbage and carrots.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J32" s="9" t="inlineStr">
@@ -8112,7 +8310,7 @@
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
@@ -8132,11 +8330,11 @@
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="8">
-        <v>46365</v>
+        <v>46355</v>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
@@ -8157,7 +8355,7 @@
       <c r="I33" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Our live herbs keep growing on the windowsill. Water them every day.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J33" s="9" t="inlineStr">
@@ -8168,7 +8366,7 @@
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr">
@@ -8188,11 +8386,11 @@
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="8">
-        <v>46366</v>
+        <v>46356</v>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F34" s="17" t="inlineStr">
@@ -8213,7 +8411,7 @@
       <c r="I34" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Garden box: six herbs standing in sleeves, and a jar of basil that keeps growing.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J34" s="9" t="inlineStr">
@@ -8224,7 +8422,7 @@
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr">
@@ -8244,11 +8442,11 @@
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="8">
-        <v>46369</v>
+        <v>46357</v>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F35" s="15" t="inlineStr">
@@ -8269,7 +8467,7 @@
       <c r="I35" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Red, yellow and green peppers — thick walls, glossy skin.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J35" s="9" t="inlineStr">
@@ -8280,7 +8478,7 @@
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
@@ -8300,11 +8498,11 @@
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="8">
-        <v>46370</v>
+        <v>46358</v>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr">
@@ -8325,7 +8523,7 @@
       <c r="I36" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Purple figs are here. Soft, sweet and delivered whole.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J36" s="9" t="inlineStr">
@@ -8336,7 +8534,7 @@
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr">
@@ -8356,11 +8554,11 @@
       </c>
       <c r="C37" s="6"/>
       <c r="D37" s="8">
-        <v>46371</v>
+        <v>46359</v>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F37" s="14" t="inlineStr">
@@ -8381,7 +8579,7 @@
       <c r="I37" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Every wrap is paper, and every piece of packaging has a second life.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J37" s="9" t="inlineStr">
@@ -8392,7 +8590,7 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr">
@@ -8412,11 +8610,11 @@
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="8">
-        <v>46372</v>
+        <v>46360</v>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F38" s="15" t="inlineStr">
@@ -8437,7 +8635,7 @@
       <c r="I38" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Pomegranates, figs, dates and persimmon. Autumn, whole and spotless.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J38" s="9" t="inlineStr">
@@ -8448,7 +8646,7 @@
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr">
@@ -8468,11 +8666,11 @@
       </c>
       <c r="C39" s="6"/>
       <c r="D39" s="8">
-        <v>46373</v>
+        <v>46361</v>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F39" s="15" t="inlineStr">
@@ -8493,7 +8691,7 @@
       <c r="I39" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Kiwis — firm, sweet-sharp and delivered whole.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J39" s="9" t="inlineStr">
@@ -8504,7 +8702,7 @@
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr">
@@ -8524,11 +8722,11 @@
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="8">
-        <v>46376</v>
+        <v>46362</v>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F40" s="15" t="inlineStr">
@@ -8549,7 +8747,7 @@
       <c r="I40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Mandarins — easy to peel, easy to share.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J40" s="9" t="inlineStr">
@@ -8560,7 +8758,7 @@
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr">
@@ -8580,11 +8778,11 @@
       </c>
       <c r="C41" s="6"/>
       <c r="D41" s="8">
-        <v>46377</v>
+        <v>46363</v>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F41" s="17" t="inlineStr">
@@ -8605,7 +8803,7 @@
       <c r="I41" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Host box arrives as a serving tray: grapes in the middle, dates, figs, strawberries and mint around it.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J41" s="9" t="inlineStr">
@@ -8616,7 +8814,7 @@
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr">
@@ -8636,11 +8834,11 @@
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="8">
-        <v>46378</v>
+        <v>46364</v>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F42" s="17" t="inlineStr">
@@ -8661,7 +8859,7 @@
       <c r="I42" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Salad Table: three lanes of greens, tomatoes and cucumbers.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J42" s="9" t="inlineStr">
@@ -8672,7 +8870,7 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr">
@@ -8692,11 +8890,11 @@
       </c>
       <c r="C43" s="6"/>
       <c r="D43" s="8">
-        <v>46379</v>
+        <v>46365</v>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
@@ -8717,7 +8915,7 @@
       <c r="I43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A crisp green apple in every lunchbox, washed and paper-wrapped.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J43" s="9" t="inlineStr">
@@ -8728,7 +8926,7 @@
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L43" s="6" t="inlineStr">
@@ -8748,11 +8946,11 @@
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="8">
-        <v>46380</v>
+        <v>46366</v>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
@@ -8773,7 +8971,7 @@
       <c r="I44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Romaine cut this morning, washed and crisp.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J44" s="9" t="inlineStr">
@@ -8784,7 +8982,7 @@
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L44" s="6" t="inlineStr">
@@ -8804,11 +9002,11 @@
       </c>
       <c r="C45" s="6"/>
       <c r="D45" s="8">
-        <v>46383</v>
+        <v>46367</v>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F45" s="15" t="inlineStr">
@@ -8829,7 +9027,7 @@
       <c r="I45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Beetroot with its leaves on — earthy, sweet and whole.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J45" s="9" t="inlineStr">
@@ -8840,7 +9038,7 @@
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L45" s="6" t="inlineStr">
@@ -8860,11 +9058,11 @@
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="8">
-        <v>46384</v>
+        <v>46368</v>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr">
@@ -8885,7 +9083,7 @@
       <c r="I46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A whole watermelon on the table is the start of every summer gathering.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J46" s="9" t="inlineStr">
@@ -8896,7 +9094,7 @@
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L46" s="6" t="inlineStr">
@@ -8916,11 +9114,11 @@
       </c>
       <c r="C47" s="6"/>
       <c r="D47" s="8">
-        <v>46385</v>
+        <v>46369</v>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr">
@@ -8941,7 +9139,7 @@
       <c r="I47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Cherries with their stems on — the bowl that empties first.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J47" s="9" t="inlineStr">
@@ -8952,7 +9150,7 @@
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L47" s="6" t="inlineStr">
@@ -8972,11 +9170,11 @@
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="8">
-        <v>46386</v>
+        <v>46370</v>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F48" s="15" t="inlineStr">
@@ -8997,7 +9195,7 @@
       <c r="I48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">December: mandarins, oranges, strawberries, broccoli, cabbage and beetroot.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J48" s="9" t="inlineStr">
@@ -9008,7 +9206,7 @@
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr">
@@ -9028,11 +9226,11 @@
       </c>
       <c r="C49" s="6"/>
       <c r="D49" s="8">
-        <v>46387</v>
+        <v>46371</v>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F49" s="14" t="inlineStr">
@@ -9053,7 +9251,7 @@
       <c r="I49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Order before noon for same-day delivery across Cairo.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J49" s="9" t="inlineStr">
@@ -9064,7 +9262,7 @@
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr">
@@ -9084,11 +9282,11 @@
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="8">
-        <v>46390</v>
+        <v>46372</v>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F50" s="13" t="inlineStr">
@@ -9109,7 +9307,7 @@
       <c r="I50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Dates and pomegranates — iftar starts with something whole.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J50" s="9" t="inlineStr">
@@ -9120,7 +9318,7 @@
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr">
@@ -9140,11 +9338,11 @@
       </c>
       <c r="C51" s="6"/>
       <c r="D51" s="8">
-        <v>46391</v>
+        <v>46373</v>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F51" s="17" t="inlineStr">
@@ -9165,7 +9363,7 @@
       <c r="I51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Salad Table box: greens, tomatoes and cucumbers in their own lanes, herbs and lemons on the side.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J51" s="9" t="inlineStr">
@@ -9176,7 +9374,7 @@
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L51" s="6" t="inlineStr">
@@ -9196,11 +9394,11 @@
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="8">
-        <v>46392</v>
+        <v>46374</v>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
@@ -9221,7 +9419,7 @@
       <c r="I52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Orange, yellow, green and purple — the easiest way to get vegetables on a child’s plate.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J52" s="9" t="inlineStr">
@@ -9232,7 +9430,7 @@
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L52" s="6" t="inlineStr">
@@ -9252,11 +9450,11 @@
       </c>
       <c r="C53" s="6"/>
       <c r="D53" s="8">
-        <v>46393</v>
+        <v>46375</v>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
@@ -9277,7 +9475,7 @@
       <c r="I53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Dill, cut the morning it ships. A little green on every plate.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J53" s="9" t="inlineStr">
@@ -9288,7 +9486,7 @@
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L53" s="6" t="inlineStr">
@@ -9308,11 +9506,11 @@
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="8">
-        <v>46394</v>
+        <v>46376</v>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F54" s="15" t="inlineStr">
@@ -9333,7 +9531,7 @@
       <c r="I54" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Guava season. You’ll smell the box before you open it.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J54" s="9" t="inlineStr">
@@ -9344,7 +9542,7 @@
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L54" s="6" t="inlineStr">
@@ -9364,11 +9562,11 @@
       </c>
       <c r="C55" s="6"/>
       <c r="D55" s="8">
-        <v>46397</v>
+        <v>46377</v>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F55" s="15" t="inlineStr">
@@ -9389,7 +9587,7 @@
       <c r="I55" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A bowl of lemons on the island changes the whole room.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J55" s="9" t="inlineStr">
@@ -9400,7 +9598,7 @@
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L55" s="6" t="inlineStr">
@@ -9420,11 +9618,11 @@
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="8">
-        <v>46398</v>
+        <v>46378</v>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F56" s="14" t="inlineStr">
@@ -9445,7 +9643,7 @@
       <c r="I56" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Crunchy red apples, washed by hand and never waxed.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J56" s="9" t="inlineStr">
@@ -9456,7 +9654,7 @@
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L56" s="6" t="inlineStr">
@@ -9476,11 +9674,11 @@
       </c>
       <c r="C57" s="6"/>
       <c r="D57" s="8">
-        <v>46399</v>
+        <v>46379</v>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F57" s="14" t="inlineStr">
@@ -9501,7 +9699,7 @@
       <c r="I57" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Eggplants picked young — glossy, firm and never bitter.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J57" s="9" t="inlineStr">
@@ -9512,7 +9710,7 @@
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L57" s="6" t="inlineStr">
@@ -9532,11 +9730,11 @@
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="8">
-        <v>46400</v>
+        <v>46380</v>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F58" s="17" t="inlineStr">
@@ -9557,7 +9755,7 @@
       <c r="I58" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Order on the site or on WhatsApp before noon for same-day delivery.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J58" s="9" t="inlineStr">
@@ -9568,7 +9766,7 @@
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr">
@@ -9588,11 +9786,11 @@
       </c>
       <c r="C59" s="6"/>
       <c r="D59" s="8">
-        <v>46401</v>
+        <v>46381</v>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F59" s="14" t="inlineStr">
@@ -9613,7 +9811,7 @@
       <c r="I59" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">If anything isn’t right, it isn’t your problem. Send a photo and we fix it.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J59" s="9" t="inlineStr">
@@ -9624,7 +9822,7 @@
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L59" s="6" t="inlineStr">
@@ -9644,11 +9842,11 @@
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="8">
-        <v>46404</v>
+        <v>46382</v>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F60" s="16" t="inlineStr">
@@ -9669,7 +9867,7 @@
       <c r="I60" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Plums at their sweetest — nothing added.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J60" s="9" t="inlineStr">
@@ -9680,7 +9878,7 @@
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L60" s="6" t="inlineStr">
@@ -9700,11 +9898,11 @@
       </c>
       <c r="C61" s="6"/>
       <c r="D61" s="8">
-        <v>46405</v>
+        <v>46383</v>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F61" s="13" t="inlineStr">
@@ -9725,7 +9923,7 @@
       <c r="I61" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Grapes — the first thing guests reach for.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J61" s="9" t="inlineStr">
@@ -9736,7 +9934,7 @@
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr">
@@ -9756,11 +9954,11 @@
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="8">
-        <v>46406</v>
+        <v>46384</v>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F62" s="13" t="inlineStr">
@@ -9781,7 +9979,7 @@
       <c r="I62" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The fruit bowl changes every week because the season does.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J62" s="9" t="inlineStr">
@@ -9792,7 +9990,7 @@
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L62" s="6" t="inlineStr">
@@ -9812,11 +10010,11 @@
       </c>
       <c r="C63" s="6"/>
       <c r="D63" s="8">
-        <v>46407</v>
+        <v>46385</v>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F63" s="14" t="inlineStr">
@@ -9837,7 +10035,7 @@
       <c r="I63" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Only the first pick of each lot makes it into a Fresh Valley box.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J63" s="9" t="inlineStr">
@@ -9848,7 +10046,7 @@
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L63" s="6" t="inlineStr">
@@ -9868,11 +10066,11 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="8">
-        <v>46408</v>
+        <v>46386</v>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F64" s="15" t="inlineStr">
@@ -9893,7 +10091,7 @@
       <c r="I64" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Peaches at their sweetest — summer in a bowl.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J64" s="9" t="inlineStr">
@@ -9904,7 +10102,7 @@
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L64" s="6" t="inlineStr">
@@ -9924,11 +10122,11 @@
       </c>
       <c r="C65" s="6"/>
       <c r="D65" s="8">
-        <v>46411</v>
+        <v>46387</v>
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F65" s="15" t="inlineStr">
@@ -9949,7 +10147,7 @@
       <c r="I65" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Persimmons, honey-sweet and delivered whole. Let them soften on the counter.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J65" s="9" t="inlineStr">
@@ -9960,7 +10158,7 @@
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L65" s="6" t="inlineStr">
@@ -9980,11 +10178,11 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="8">
-        <v>46412</v>
+        <v>46388</v>
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F66" s="15" t="inlineStr">
@@ -10005,7 +10203,7 @@
       <c r="I66" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">January: oranges, mandarins, strawberries, guava, cauliflower and spinach.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J66" s="9" t="inlineStr">
@@ -10016,7 +10214,7 @@
       </c>
       <c r="K66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L66" s="6" t="inlineStr">
@@ -10036,11 +10234,11 @@
       </c>
       <c r="C67" s="6"/>
       <c r="D67" s="8">
-        <v>46413</v>
+        <v>46389</v>
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F67" s="14" t="inlineStr">
@@ -10061,7 +10259,7 @@
       <c r="I67" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Nothing waits in a warehouse. You order, we pick, it ships the same day.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J67" s="9" t="inlineStr">
@@ -10072,7 +10270,7 @@
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr">
@@ -10092,11 +10290,11 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="8">
-        <v>46414</v>
+        <v>46390</v>
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F68" s="13" t="inlineStr">
@@ -10117,7 +10315,7 @@
       <c r="I68" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Grapes, pomegranates and figs — made for long tables.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J68" s="9" t="inlineStr">
@@ -10128,7 +10326,7 @@
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr">
@@ -10148,11 +10346,11 @@
       </c>
       <c r="C69" s="6"/>
       <c r="D69" s="8">
-        <v>46415</v>
+        <v>46391</v>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F69" s="13" t="inlineStr">
@@ -10174,7 +10372,7 @@
       <c r="I69" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Build a fruit tray in four steps: grapes in the middle, dates and figs around them, colour from strawberries and pomegranates, mint to finish. Save it for your next gathering.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J69" s="9" t="inlineStr">
@@ -10185,7 +10383,7 @@
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L69" s="6" t="inlineStr">
@@ -10205,11 +10403,11 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="8">
-        <v>46418</v>
+        <v>46392</v>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F70" s="13" t="inlineStr">
@@ -10231,7 +10429,7 @@
       <c r="I70" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A box for every occasion: The Host for a housewarming, The Orchard to say thank you, The Garden for a new kitchen, The Market to say get well soon.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J70" s="9" t="inlineStr">
@@ -10242,7 +10440,7 @@
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr">
@@ -10262,11 +10460,11 @@
       </c>
       <c r="C71" s="6"/>
       <c r="D71" s="8">
-        <v>46419</v>
+        <v>46393</v>
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F71" s="16" t="inlineStr">
@@ -10287,7 +10485,7 @@
       <c r="I71" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Rosemary, cut the morning it ships. The smell of a slow Friday.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J71" s="9" t="inlineStr">
@@ -10298,7 +10496,7 @@
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr">
@@ -10318,11 +10516,11 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="8">
-        <v>46420</v>
+        <v>46394</v>
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F72" s="14" t="inlineStr">
@@ -10343,7 +10541,7 @@
       <c r="I72" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Apples, pears, oranges, peaches — every one Grade A, every one whole.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J72" s="9" t="inlineStr">
@@ -10354,7 +10552,7 @@
       </c>
       <c r="K72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L72" s="6" t="inlineStr">
@@ -10374,11 +10572,11 @@
       </c>
       <c r="C73" s="6"/>
       <c r="D73" s="8">
-        <v>46421</v>
+        <v>46395</v>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F73" s="13" t="inlineStr">
@@ -10400,7 +10598,7 @@
       <c r="I73" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Every group has one. Tag the friend who always hosts — the next box might be on us.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J73" s="9" t="inlineStr">
@@ -10411,7 +10609,7 @@
       </c>
       <c r="K73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L73" s="6" t="inlineStr">
@@ -10431,11 +10629,11 @@
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="8">
-        <v>46422</v>
+        <v>46396</v>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F74" s="13" t="inlineStr">
@@ -10457,7 +10655,7 @@
       <c r="I74" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">One fruit for the middle of your tray — 1, 2, 3 or 4? Comment your number.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J74" s="9" t="inlineStr">
@@ -10468,7 +10666,7 @@
       </c>
       <c r="K74" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L74" s="6" t="inlineStr">
@@ -10488,11 +10686,11 @@
       </c>
       <c r="C75" s="6"/>
       <c r="D75" s="8">
-        <v>46425</v>
+        <v>46397</v>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F75" s="14" t="inlineStr">
@@ -10513,7 +10711,7 @@
       <c r="I75" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Green beans picked young — they snap, they don’t bend.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J75" s="9" t="inlineStr">
@@ -10524,7 +10722,7 @@
       </c>
       <c r="K75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L75" s="6" t="inlineStr">
@@ -10544,11 +10742,11 @@
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="8">
-        <v>46426</v>
+        <v>46398</v>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F76" s="17" t="inlineStr">
@@ -10569,7 +10767,7 @@
       <c r="I76" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Fruit and vegetables for the whole week, delivered the day they’re picked.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J76" s="9" t="inlineStr">
@@ -10580,7 +10778,7 @@
       </c>
       <c r="K76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L76" s="6" t="inlineStr">
@@ -10600,11 +10798,11 @@
       </c>
       <c r="C77" s="6"/>
       <c r="D77" s="8">
-        <v>46427</v>
+        <v>46399</v>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F77" s="17" t="inlineStr">
@@ -10625,7 +10823,7 @@
       <c r="I77" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The carry box: a handle on top and a box of whole fruit inside. Ask about gift notes on WhatsApp.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J77" s="9" t="inlineStr">
@@ -10636,7 +10834,7 @@
       </c>
       <c r="K77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L77" s="6" t="inlineStr">
@@ -10656,11 +10854,11 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="8">
-        <v>46428</v>
+        <v>46400</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F78" s="15" t="inlineStr">
@@ -10681,7 +10879,7 @@
       <c r="I78" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Oranges, lemons and mandarins — winter in colour.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J78" s="9" t="inlineStr">
@@ -10692,7 +10890,7 @@
       </c>
       <c r="K78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L78" s="6" t="inlineStr">
@@ -10712,11 +10910,11 @@
       </c>
       <c r="C79" s="6"/>
       <c r="D79" s="8">
-        <v>46429</v>
+        <v>46401</v>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F79" s="15" t="inlineStr">
@@ -10738,7 +10936,7 @@
       <c r="I79" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Mango team or strawberry team? Tell us in the comments.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J79" s="9" t="inlineStr">
@@ -10749,7 +10947,7 @@
       </c>
       <c r="K79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L79" s="6" t="inlineStr">
@@ -10769,11 +10967,11 @@
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="8">
-        <v>46432</v>
+        <v>46402</v>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F80" s="15" t="inlineStr">
@@ -10795,7 +10993,7 @@
       <c r="I80" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Winter, month by month: what’s at its best in December, January and February. Swipe and save.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J80" s="9" t="inlineStr">
@@ -10806,7 +11004,7 @@
       </c>
       <c r="K80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L80" s="6" t="inlineStr">
@@ -10826,11 +11024,11 @@
       </c>
       <c r="C81" s="6"/>
       <c r="D81" s="8">
-        <v>46433</v>
+        <v>46403</v>
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F81" s="14" t="inlineStr">
@@ -10852,7 +11050,7 @@
       <c r="I81" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Three checks before anything leaves the farm: picked today, colour and skin, taste. Swipe through the A check.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J81" s="9" t="inlineStr">
@@ -10863,7 +11061,7 @@
       </c>
       <c r="K81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L81" s="6" t="inlineStr">
@@ -10883,11 +11081,11 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="8">
-        <v>46434</v>
+        <v>46404</v>
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F82" s="13" t="inlineStr">
@@ -10909,7 +11107,7 @@
       <c r="I82" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Save this for your next gathering — and send it to whoever is hosting.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J82" s="9" t="inlineStr">
@@ -10920,7 +11118,7 @@
       </c>
       <c r="K82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L82" s="6" t="inlineStr">
@@ -10940,11 +11138,11 @@
       </c>
       <c r="C83" s="6"/>
       <c r="D83" s="8">
-        <v>46435</v>
+        <v>46405</v>
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F83" s="13" t="inlineStr">
@@ -10965,7 +11163,7 @@
       <c r="I83" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Medjool dates — soft, rich and the first thing on every table.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J83" s="9" t="inlineStr">
@@ -10976,7 +11174,7 @@
       </c>
       <c r="K83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L83" s="6" t="inlineStr">
@@ -10996,11 +11194,11 @@
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="8">
-        <v>46436</v>
+        <v>46406</v>
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F84" s="14" t="inlineStr">
@@ -11021,7 +11219,7 @@
       <c r="I84" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Lemons with thin skin and plenty of juice, washed and ready.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J84" s="9" t="inlineStr">
@@ -11032,7 +11230,7 @@
       </c>
       <c r="K84" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L84" s="6" t="inlineStr">
@@ -11052,11 +11250,11 @@
       </c>
       <c r="C85" s="6"/>
       <c r="D85" s="8">
-        <v>46439</v>
+        <v>46407</v>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
@@ -11078,7 +11276,7 @@
       <c r="I85" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Sweet or sour? Comment your side.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J85" s="9" t="inlineStr">
@@ -11089,7 +11287,7 @@
       </c>
       <c r="K85" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L85" s="6" t="inlineStr">
@@ -11109,11 +11307,11 @@
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="8">
-        <v>46440</v>
+        <v>46408</v>
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F86" s="17" t="inlineStr">
@@ -11135,7 +11333,7 @@
       <c r="I86" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Fill the bag — what goes in first? Tell us in the comments.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J86" s="9" t="inlineStr">
@@ -11146,7 +11344,7 @@
       </c>
       <c r="K86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L86" s="6" t="inlineStr">
@@ -11166,11 +11364,11 @@
       </c>
       <c r="C87" s="6"/>
       <c r="D87" s="8">
-        <v>46441</v>
+        <v>46409</v>
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
@@ -11191,7 +11389,7 @@
       <c r="I87" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A handful of spinach a day — tender, washed and cut the morning it ships.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J87" s="9" t="inlineStr">
@@ -11202,7 +11400,7 @@
       </c>
       <c r="K87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L87" s="6" t="inlineStr">
@@ -11222,11 +11420,11 @@
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="8">
-        <v>46442</v>
+        <v>46410</v>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F88" s="15" t="inlineStr">
@@ -11247,7 +11445,7 @@
       <c r="I88" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Apricot season is short. Velvet skin, fragrant and delivered whole.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J88" s="9" t="inlineStr">
@@ -11258,7 +11456,7 @@
       </c>
       <c r="K88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L88" s="6" t="inlineStr">
@@ -11278,11 +11476,11 @@
       </c>
       <c r="C89" s="6"/>
       <c r="D89" s="8">
-        <v>46443</v>
+        <v>46411</v>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F89" s="14" t="inlineStr">
@@ -11303,7 +11501,7 @@
       <c r="I89" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Every piece arrives washed by hand and wrapped in paper — ready to serve.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J89" s="9" t="inlineStr">
@@ -11314,7 +11512,7 @@
       </c>
       <c r="K89" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L89" s="6" t="inlineStr">
@@ -11334,11 +11532,11 @@
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="8">
-        <v>46446</v>
+        <v>46412</v>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F90" s="17" t="inlineStr">
@@ -11360,7 +11558,7 @@
       <c r="I90" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">One box, three sizes: Petite serves 2–4, Signature 6–8, Grand 10–12.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J90" s="9" t="inlineStr">
@@ -11371,7 +11569,7 @@
       </c>
       <c r="K90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L90" s="6" t="inlineStr">
@@ -11391,11 +11589,11 @@
       </c>
       <c r="C91" s="6"/>
       <c r="D91" s="8">
-        <v>46447</v>
+        <v>46413</v>
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F91" s="17" t="inlineStr">
@@ -11417,7 +11615,7 @@
       <c r="I91" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Orchard, the Market, the Garden, the Salad Table or the Host — which box are you? Comment yours.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J91" s="9" t="inlineStr">
@@ -11428,7 +11626,7 @@
       </c>
       <c r="K91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L91" s="6" t="inlineStr">
@@ -11448,11 +11646,11 @@
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="8">
-        <v>46448</v>
+        <v>46414</v>
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F92" s="16" t="inlineStr">
@@ -11473,7 +11671,7 @@
       <c r="I92" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Carrots, cucumbers and radishes — the crunchiest snack in the house.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J92" s="9" t="inlineStr">
@@ -11484,7 +11682,7 @@
       </c>
       <c r="K92" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L92" s="6" t="inlineStr">
@@ -11504,11 +11702,11 @@
       </c>
       <c r="C93" s="6"/>
       <c r="D93" s="8">
-        <v>46449</v>
+        <v>46415</v>
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F93" s="16" t="inlineStr">
@@ -11530,7 +11728,7 @@
       <c r="I93" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Herbs last a week if you trim the stems, stand them in water and cover them loosely in the fridge. Basil stays on the counter.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J93" s="9" t="inlineStr">
@@ -11541,7 +11739,7 @@
       </c>
       <c r="K93" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L93" s="6" t="inlineStr">
@@ -11561,11 +11759,11 @@
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="8">
-        <v>46450</v>
+        <v>46416</v>
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F94" s="14" t="inlineStr">
@@ -11587,7 +11785,7 @@
       <c r="I94" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Which one would you pick? Trick question — they’re all Grade A.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J94" s="9" t="inlineStr">
@@ -11598,7 +11796,7 @@
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L94" s="6" t="inlineStr">
@@ -11618,11 +11816,11 @@
       </c>
       <c r="C95" s="6"/>
       <c r="D95" s="8">
-        <v>46453</v>
+        <v>46417</v>
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F95" s="15" t="inlineStr">
@@ -11643,7 +11841,7 @@
       <c r="I95" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Mandarins — easy to peel, easy to share.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J95" s="9" t="inlineStr">
@@ -11654,7 +11852,7 @@
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L95" s="6" t="inlineStr">
@@ -11674,11 +11872,11 @@
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="8">
-        <v>46454</v>
+        <v>46418</v>
       </c>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F96" s="13" t="inlineStr">
@@ -11699,7 +11897,7 @@
       <c r="I96" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Hosting this week? We’ve got the table covered.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J96" s="9" t="inlineStr">
@@ -11710,7 +11908,7 @@
       </c>
       <c r="K96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L96" s="6" t="inlineStr">
@@ -11730,11 +11928,11 @@
       </c>
       <c r="C97" s="6"/>
       <c r="D97" s="8">
-        <v>46455</v>
+        <v>46419</v>
       </c>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F97" s="14" t="inlineStr">
@@ -11756,7 +11954,7 @@
       <c r="I97" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">What do you think makes fruit Grade A? Comment your guess — we reply to every one, and share the answer on Friday.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J97" s="9" t="inlineStr">
@@ -11767,7 +11965,7 @@
       </c>
       <c r="K97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #ClassA #HandGraded #متنقي_بالإيد</t>
+          <t xml:space="preserve">#FreshValley #ClassA #HandGraded #FreshProduce</t>
         </is>
       </c>
       <c r="L97" s="6" t="inlineStr">
@@ -11787,11 +11985,11 @@
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="8">
-        <v>46456</v>
+        <v>46420</v>
       </c>
       <c r="E98" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F98" s="17" t="inlineStr">
@@ -11812,7 +12010,7 @@
       <c r="I98" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The gift that never ends up in a cupboard. Send a box today.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J98" s="9" t="inlineStr">
@@ -11823,7 +12021,7 @@
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L98" s="6" t="inlineStr">
@@ -11843,11 +12041,11 @@
       </c>
       <c r="C99" s="6"/>
       <c r="D99" s="8">
-        <v>46457</v>
+        <v>46421</v>
       </c>
       <c r="E99" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
@@ -11868,7 +12066,7 @@
       <c r="I99" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Radishes with their leaves on — peppery, crisp and picked today.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J99" s="9" t="inlineStr">
@@ -11879,7 +12077,7 @@
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L99" s="6" t="inlineStr">
@@ -11899,11 +12097,11 @@
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="8">
-        <v>46460</v>
+        <v>46422</v>
       </c>
       <c r="E100" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Thu · 9:00 pm</t>
         </is>
       </c>
       <c r="F100" s="15" t="inlineStr">
@@ -11925,7 +12123,7 @@
       <c r="I100" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Pick your winter three — comment them below.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J100" s="9" t="inlineStr">
@@ -11936,7 +12134,7 @@
       </c>
       <c r="K100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #InSeason #فاكهة_الموسم #WholeProduce</t>
+          <t xml:space="preserve">#FreshValley #InSeason #WholeProduce #EatSeasonal</t>
         </is>
       </c>
       <c r="L100" s="6" t="inlineStr">
@@ -11956,11 +12154,11 @@
       </c>
       <c r="C101" s="6"/>
       <c r="D101" s="8">
-        <v>46461</v>
+        <v>46423</v>
       </c>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Fri · 1:30 pm</t>
         </is>
       </c>
       <c r="F101" s="17" t="inlineStr">
@@ -11981,7 +12179,7 @@
       <c r="I101" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">The Host box: grapes, dates, figs, strawberries and mint — the whole table in one box.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J101" s="9" t="inlineStr">
@@ -11992,7 +12190,7 @@
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L101" s="6" t="inlineStr">
@@ -12012,11 +12210,11 @@
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="8">
-        <v>46462</v>
+        <v>46424</v>
       </c>
       <c r="E102" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sat · 12:00 pm</t>
         </is>
       </c>
       <c r="F102" s="13" t="inlineStr">
@@ -12037,7 +12235,7 @@
       <c r="I102" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Grapes, figs, pomegranates and dates — a full table in four.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J102" s="9" t="inlineStr">
@@ -12048,7 +12246,7 @@
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L102" s="6" t="inlineStr">
@@ -12068,11 +12266,11 @@
       </c>
       <c r="C103" s="6"/>
       <c r="D103" s="8">
-        <v>46463</v>
+        <v>46425</v>
       </c>
       <c r="E103" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Sun · 8:30 pm</t>
         </is>
       </c>
       <c r="F103" s="13" t="inlineStr">
@@ -12093,7 +12291,7 @@
       <c r="I103" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A whole pineapple, crown on — the centrepiece every table needs.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J103" s="9" t="inlineStr">
@@ -12104,7 +12302,7 @@
       </c>
       <c r="K103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L103" s="6" t="inlineStr">
@@ -12124,11 +12322,11 @@
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="8">
-        <v>46464</v>
+        <v>46426</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:00 pm</t>
+          <t xml:space="preserve">Mon · 8:30 pm</t>
         </is>
       </c>
       <c r="F104" s="17" t="inlineStr">
@@ -12149,7 +12347,7 @@
       <c r="I104" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Packed this morning, wrapped in paper, at your door today.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J104" s="9" t="inlineStr">
@@ -12160,7 +12358,7 @@
       </c>
       <c r="K104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTableBox #بوكس_السفرة #Gifting</t>
+          <t xml:space="preserve">#FreshValley #TheTableBox #GiftBox #Gifting</t>
         </is>
       </c>
       <c r="L104" s="6" t="inlineStr">
@@ -12180,11 +12378,11 @@
       </c>
       <c r="C105" s="6"/>
       <c r="D105" s="8">
-        <v>46467</v>
+        <v>46427</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Tue · 8:30 pm</t>
         </is>
       </c>
       <c r="F105" s="13" t="inlineStr">
@@ -12206,7 +12404,7 @@
       <c r="I105" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Dates or figs — which one makes your table? Comment A or B.
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J105" s="9" t="inlineStr">
@@ -12217,7 +12415,7 @@
       </c>
       <c r="K105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #TheTable #Hosting #سفرة #ضيافة</t>
+          <t xml:space="preserve">#FreshValley #TheTable #Hosting #FruitPlatter</t>
         </is>
       </c>
       <c r="L105" s="6" t="inlineStr">
@@ -12237,11 +12435,11 @@
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="8">
-        <v>46468</v>
+        <v>46428</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8:30 pm</t>
+          <t xml:space="preserve">Wed · 8:30 pm</t>
         </is>
       </c>
       <c r="F106" s="16" t="inlineStr">
@@ -12263,7 +12461,7 @@
       <c r="I106" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">True or false: basil belongs in the fridge? Comment your answer — we’ll reply with the right one. (Hint: it loves a sunny windowsill.)
-Order before noon — at your door today. Link in bio.</t>
+Order before noon for same-day delivery. Link in bio.</t>
         </is>
       </c>
       <c r="J106" s="9" t="inlineStr">
@@ -12274,7 +12472,7 @@
       </c>
       <c r="K106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">#FreshValley #فريش_فالي #LivingWell #EatMorePlants #أكل_صحي</t>
+          <t xml:space="preserve">#FreshValley #LivingWell #EatMorePlants #FreshHerbs</t>
         </is>
       </c>
       <c r="L106" s="6" t="inlineStr">
@@ -12572,11 +12770,11 @@
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="8">
-        <v>46412</v>
+        <v>46327</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -12606,11 +12804,11 @@
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="8">
-        <v>46413</v>
+        <v>46330</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -12640,11 +12838,11 @@
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="8">
-        <v>46415</v>
+        <v>46334</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -12674,11 +12872,11 @@
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="8">
-        <v>46416</v>
+        <v>46337</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
@@ -12708,11 +12906,11 @@
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="8">
-        <v>46419</v>
+        <v>46341</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -12742,11 +12940,11 @@
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="8">
-        <v>46420</v>
+        <v>46344</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -12776,11 +12974,11 @@
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="8">
-        <v>46422</v>
+        <v>46348</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -12810,11 +13008,11 @@
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="8">
-        <v>46423</v>
+        <v>46351</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -12844,11 +13042,11 @@
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="8">
-        <v>46426</v>
+        <v>46355</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -12878,11 +13076,11 @@
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="8">
-        <v>46427</v>
+        <v>46358</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -12912,11 +13110,11 @@
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="8">
-        <v>46429</v>
+        <v>46362</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -12946,11 +13144,11 @@
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="8">
-        <v>46430</v>
+        <v>46365</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
@@ -12980,11 +13178,11 @@
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="8">
-        <v>46433</v>
+        <v>46369</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
@@ -13014,11 +13212,11 @@
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="8">
-        <v>46434</v>
+        <v>46372</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
@@ -13048,11 +13246,11 @@
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="8">
-        <v>46436</v>
+        <v>46376</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
@@ -13082,11 +13280,11 @@
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="8">
-        <v>46437</v>
+        <v>46379</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
@@ -13116,11 +13314,11 @@
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="8">
-        <v>46440</v>
+        <v>46383</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
@@ -13150,11 +13348,11 @@
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="8">
-        <v>46441</v>
+        <v>46386</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
@@ -13184,11 +13382,11 @@
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="8">
-        <v>46443</v>
+        <v>46390</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E23" s="16" t="inlineStr">
@@ -13218,11 +13416,11 @@
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="8">
-        <v>46444</v>
+        <v>46393</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E24" s="16" t="inlineStr">
@@ -13252,11 +13450,11 @@
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="8">
-        <v>46447</v>
+        <v>46397</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E25" s="16" t="inlineStr">
@@ -13286,11 +13484,11 @@
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="8">
-        <v>46448</v>
+        <v>46400</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E26" s="16" t="inlineStr">
@@ -13320,11 +13518,11 @@
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="8">
-        <v>46450</v>
+        <v>46404</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E27" s="16" t="inlineStr">
@@ -13354,11 +13552,11 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="8">
-        <v>46451</v>
+        <v>46407</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E28" s="16" t="inlineStr">
@@ -13388,11 +13586,11 @@
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="8">
-        <v>46454</v>
+        <v>46411</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E29" s="17" t="inlineStr">
@@ -13422,11 +13620,11 @@
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="8">
-        <v>46455</v>
+        <v>46414</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
@@ -13456,11 +13654,11 @@
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="8">
-        <v>46457</v>
+        <v>46418</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E31" s="17" t="inlineStr">
@@ -13490,11 +13688,11 @@
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="8">
-        <v>46458</v>
+        <v>46421</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E32" s="17" t="inlineStr">
@@ -13524,11 +13722,11 @@
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="8">
-        <v>46461</v>
+        <v>46425</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">11:00 am</t>
         </is>
       </c>
       <c r="E33" s="17" t="inlineStr">
@@ -13558,11 +13756,11 @@
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="8">
-        <v>46462</v>
+        <v>46428</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7:00 pm</t>
+          <t xml:space="preserve">5:00 pm</t>
         </is>
       </c>
       <c r="E34" s="17" t="inlineStr">
@@ -14115,7 +14313,7 @@
   <sheetPr>
     <tabColor rgb="FFDCE3D2"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -14202,17 +14400,17 @@
       <c r="B6" s="6"/>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">circle sticker</t>
+          <t xml:space="preserve">circle sticker 2c</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round seal sticker</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/circle-sticker.png</t>
+          <t xml:space="preserve">pack2/png/circle-sticker-2c.png</t>
         </is>
       </c>
     </row>
@@ -14223,17 +14421,17 @@
       <c r="B7" s="6"/>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">drawstring</t>
+          <t xml:space="preserve">circle sticker</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cotton drawstring bag</t>
+          <t xml:space="preserve">Round seal sticker</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/drawstring.png</t>
+          <t xml:space="preserve">pack2/png/circle-sticker.png</t>
         </is>
       </c>
     </row>
@@ -14244,17 +14442,17 @@
       <c r="B8" s="6"/>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">lid garden</t>
+          <t xml:space="preserve">drawstring</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box lid (top face)</t>
+          <t xml:space="preserve">Cotton drawstring bag</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/lid-garden.png</t>
+          <t xml:space="preserve">pack2/png/drawstring.png</t>
         </is>
       </c>
     </row>
@@ -14265,17 +14463,17 @@
       <c r="B9" s="6"/>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">lid host</t>
+          <t xml:space="preserve">insert garden</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box lid (top face)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/lid-host.png</t>
+          <t xml:space="preserve">pack2/png/insert-garden.png</t>
         </is>
       </c>
     </row>
@@ -14286,17 +14484,17 @@
       <c r="B10" s="6"/>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">lid market</t>
+          <t xml:space="preserve">insert host</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box lid (top face)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/lid-market.png</t>
+          <t xml:space="preserve">pack2/png/insert-host.png</t>
         </is>
       </c>
     </row>
@@ -14307,17 +14505,17 @@
       <c r="B11" s="6"/>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">lid orchard</t>
+          <t xml:space="preserve">insert market</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box lid (top face)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/lid-orchard.png</t>
+          <t xml:space="preserve">pack2/png/insert-market.png</t>
         </is>
       </c>
     </row>
@@ -14328,17 +14526,17 @@
       <c r="B12" s="6"/>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">lid salad</t>
+          <t xml:space="preserve">insert orchard</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box lid (top face)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/lid-salad.png</t>
+          <t xml:space="preserve">pack2/png/insert-orchard.png</t>
         </is>
       </c>
     </row>
@@ -14349,143 +14547,143 @@
       <c r="B13" s="6"/>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">paper bag</t>
+          <t xml:space="preserve">insert salad</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paper grocery bag</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/paper-bag.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="60" customHeight="1">
+          <t xml:space="preserve">pack2/png/insert-salad.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="139.5" customHeight="1">
       <c r="A14" s="7">
         <v>10</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">punnet band</t>
+          <t xml:space="preserve">lid garden</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strawberry punnet band</t>
+          <t xml:space="preserve">Box lid (top face)</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/punnet-band.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="129" customHeight="1">
+          <t xml:space="preserve">pack2/png/lid-garden.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="139.5" customHeight="1">
       <c r="A15" s="7">
         <v>11</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ship label</t>
+          <t xml:space="preserve">lid host</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shipping label on every box</t>
+          <t xml:space="preserve">Box lid (top face)</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/ship-label.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+          <t xml:space="preserve">pack2/png/lid-host.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="139.5" customHeight="1">
       <c r="A16" s="7">
         <v>12</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">side garden</t>
+          <t xml:space="preserve">lid market</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box long side</t>
+          <t xml:space="preserve">Box lid (top face)</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/side-garden.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1">
+          <t xml:space="preserve">pack2/png/lid-market.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="139.5" customHeight="1">
       <c r="A17" s="7">
         <v>13</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">side host</t>
+          <t xml:space="preserve">lid orchard</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box long side</t>
+          <t xml:space="preserve">Box lid (top face)</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/side-host.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
+          <t xml:space="preserve">pack2/png/lid-orchard.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="139.5" customHeight="1">
       <c r="A18" s="7">
         <v>14</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">side market</t>
+          <t xml:space="preserve">lid salad</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box long side</t>
+          <t xml:space="preserve">Box lid (top face)</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/side-market.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="60" customHeight="1">
+          <t xml:space="preserve">pack2/png/lid-salad.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="139.5" customHeight="1">
       <c r="A19" s="7">
         <v>15</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">side orchard</t>
+          <t xml:space="preserve">paper bag</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box long side</t>
+          <t xml:space="preserve">Paper grocery bag</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/side-orchard.png</t>
+          <t xml:space="preserve">pack2/png/paper-bag.png</t>
         </is>
       </c>
     </row>
@@ -14496,36 +14694,162 @@
       <c r="B20" s="6"/>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">side salad</t>
+          <t xml:space="preserve">punnet band</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box long side</t>
+          <t xml:space="preserve">Strawberry punnet band</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack2/png/side-salad.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="139.5" customHeight="1">
+          <t xml:space="preserve">pack2/png/punnet-band.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="129" customHeight="1">
       <c r="A21" s="7">
         <v>17</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">ship label</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipping label on every box</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pack2/png/ship-label.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70.5" customHeight="1">
+      <c r="A22" s="7">
+        <v>18</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">side garden</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box long side</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pack2/png/side-garden.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="70.5" customHeight="1">
+      <c r="A23" s="7">
+        <v>19</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">side host</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box long side</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pack2/png/side-host.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="70.5" customHeight="1">
+      <c r="A24" s="7">
+        <v>20</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">side market</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box long side</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pack2/png/side-market.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="70.5" customHeight="1">
+      <c r="A25" s="7">
+        <v>21</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">side orchard</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box long side</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pack2/png/side-orchard.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="70.5" customHeight="1">
+      <c r="A26" s="7">
+        <v>22</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">side salad</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box long side</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pack2/png/side-salad.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="139.5" customHeight="1">
+      <c r="A27" s="7">
+        <v>23</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">tote dark</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Canvas tote, front</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">pack2/png/tote-dark.png</t>
         </is>

</xml_diff>